<commit_message>
docs: la lista de las 54 regenerada con los rellenos que si se pintan
La regeneracion de las 16:06 se hizo con el script anterior al arreglo de
rellenos (que entro a las 16:58): carrera de tiempos, no fallo del arreglo.
Regenerada y verificada celda por celda: cabecera azul, veredictos rojo/verde
y observaciones ambar llevan fg y bg con el mismo color.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/REVISION-54-areas-sobre-el-canal.xlsx
+++ b/docs/REVISION-54-areas-sobre-el-canal.xlsx
@@ -57,26 +57,31 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FF1F4E79"/>
+        <bgColor rgb="FF1F4E79"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFCE4E4"/>
+        <bgColor rgb="FFFCE4E4"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFF2F2F2"/>
+        <bgColor rgb="FFF2F2F2"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFE2EFDA"/>
+        <bgColor rgb="FFE2EFDA"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFFF2CC"/>
+        <bgColor rgb="FFFFF2CC"/>
       </patternFill>
     </fill>
   </fills>
@@ -3156,21 +3161,21 @@
     <row r="4">
       <c r="B4" s="9" t="inlineStr">
         <is>
-          <t>QUÉ PASA CON ESTAS FICHAS</t>
+          <t>EL PROBLEMA</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="B5" s="8" t="inlineStr">
         <is>
-          <t>En las 54, el área total, el área con riego y el área sin riego traen el mismo número. Es imposible: un predio no puede estar entero con riego y entero sin riego a la vez. Son 56,38 ha contadas dos veces, y son la única causa de que la superficie del padrón no cuadre.</t>
+          <t>En estas fichas el área total, el área con riego y el área sin riego traen el mismo número. Eso hace que el predio se cuente dos veces —entero con riego y entero sin riego— y son 56,38 ha de más en la superficie del padrón.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="B6" s="8" t="inlineStr">
         <is>
-          <t>Todas son del mismo levantamiento, entre el 24 y el 30 de julio de 2026.</t>
+          <t>Todas son del mismo levantamiento, del 24 al 30 de julio de 2026.</t>
         </is>
       </c>
     </row>
@@ -3180,52 +3185,52 @@
     <row r="8">
       <c r="B8" s="9" t="inlineStr">
         <is>
-          <t>CÓMO SE DECIDIÓ CUÁL DE LOS DOS CAMPOS SOBRA</t>
+          <t>EL CRITERIO: LA POSICIÓN RESPECTO AL CANAL</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="B9" s="8" t="inlineStr">
         <is>
-          <t>Armando lo resolvió el 12 de agosto mirando las fichas en el mapa: en PAMBAMARCA «casi todos los adicionales están sobre el canal, no tienen riego»; en CHAUPIESTANCIA «todos están bajo el canal, deben tener riego».</t>
+          <t>El canal riega por gravedad: un predio que queda por encima del canal no recibe agua, y uno que queda por debajo sí. Para clasificar cada ficha se comparó su cota con la de los 15 predios regantes más cercanos; si está más de 25 m por encima, quedó sobre el canal.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="B10" s="8" t="inlineStr">
         <is>
-          <t>El canal riega por gravedad, así que lo que queda por encima de su cota no recibe agua aunque esté al lado. Para aplicar ese criterio ficha por ficha se compara la cota de cada predio con la de las 15 fichas regantes más cercanas: si está más de 25 m por encima, quedó sobre el canal.</t>
+          <t>Resultado: Pambamarca 22 sobre y 8 bajo; Chaupiestancia 1 sobre y 17 bajo; Pucará 2 sobre; Chinchinloma 1 bajo; sin comunidad 2 sobre y 1 bajo.</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="B11" s="8" t="inlineStr">
-        <is>
-          <t>El resultado reproduce lo que dijo Armando sin habérselo indicado al programa: Pambamarca 22 sobre y 8 bajo; Chaupiestancia 1 sobre y 17 bajo.</t>
-        </is>
-      </c>
+      <c r="B11" s="8" t="inlineStr"/>
     </row>
     <row r="12">
-      <c r="B12" s="8" t="inlineStr"/>
+      <c r="B12" s="9" t="inlineStr">
+        <is>
+          <t>QUÉ HAY QUE HACER CON ESTA HOJA</t>
+        </is>
+      </c>
     </row>
     <row r="13">
-      <c r="B13" s="9" t="inlineStr">
-        <is>
-          <t>QUÉ HAY QUE REVISAR</t>
+      <c r="B13" s="8" t="inlineStr">
+        <is>
+          <t>1. Revisar en el mapa las filas con la observación «Cerca del límite»: están a pocos metros del corte de los 25 m y son las únicas dudosas.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="B14" s="8" t="inlineStr">
         <is>
-          <t>Las filas con observación en ámbar están cerca del límite de los 25 m: son las que conviene mirar en el mapa antes de aplicar nada. El resto tiene un margen claro.</t>
+          <t>2. Marcar la columna ¿CORRECTO? con SÍ o NO en las que se revisen.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="B15" s="8" t="inlineStr">
         <is>
-          <t>Marcar en la columna ¿CORRECTO? con SÍ o NO. Con eso se aplica la corrección.</t>
+          <t>3. Con la lista validada se aplica la corrección.</t>
         </is>
       </c>
     </row>
@@ -3235,14 +3240,14 @@
     <row r="17">
       <c r="B17" s="9" t="inlineStr">
         <is>
-          <t>QUÉ PASA DESPUÉS</t>
+          <t>QUÉ HACE LA CORRECCIÓN</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="B18" s="8" t="inlineStr">
         <is>
-          <t>A las que quedan SOBRE el canal se les pone el área con riego en cero; a las que quedan BAJO, el área sin riego. En los dos casos el área total del predio no se toca, porque el catastro la confirma.</t>
+          <t>A las que quedan SOBRE el canal se les pone el área con riego en cero; a las que quedan BAJO, el área sin riego en cero. El área total del predio no se toca en ningún caso: el polígono del catastro la confirma.</t>
         </is>
       </c>
     </row>

</xml_diff>